<commit_message>
Location for Tutorial 11
</commit_message>
<xml_diff>
--- a/classes.xlsx
+++ b/classes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tobychan/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCAE4E4C-69F4-E34C-84C8-7F8E2A37E1D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{780156C0-F4EE-1946-A20A-58CC4DC9A7FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22240" yWindow="500" windowWidth="16160" windowHeight="17500" xr2:uid="{3187FA12-9468-D749-A226-2B99DCD8678D}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1690" uniqueCount="352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1691" uniqueCount="352">
   <si>
     <t>start</t>
   </si>
@@ -9495,6 +9495,9 @@
       <c r="G286" s="1" t="s">
         <v>339</v>
       </c>
+      <c r="I286" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="287" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A287" s="1" t="s">

</xml_diff>